<commit_message>
base et jouer des cartes!!!!!
</commit_message>
<xml_diff>
--- a/Feuille de calcul sans titre.xlsx
+++ b/Feuille de calcul sans titre.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivi\OneDrive\Documents\4A_INFO\S1\Projet_Hero_Realms\Projet_Hero_Realms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CE385C8-E014-4A8A-941F-0D789C39DD5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08CF8561-EB2F-4EED-AE12-CB5184CD52C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>